<commit_message>
Mise à jour du dashboard et du code
</commit_message>
<xml_diff>
--- a/Gas storages.xlsx
+++ b/Gas storages.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\gvaps1\USR6\CHGE\desktop\EUA dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B69DC755-AD3B-4F33-8028-84BC7992DDC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D413E69-884F-4DA6-A609-13F72EEED2D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F907BD33-5E94-4CC9-9082-BD4BC09FA10B}"/>
   </bookViews>
@@ -186,56 +186,56 @@
       </tp>
     </main>
     <main first="bloomberg.rtd">
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>Last Price</v>
         <stp/>
         <stp>##V3_BFIELDINFOV12</stp>
         <stp>[Gas storages.xlsx]Prices!R5C2</stp>
         <stp>PX_LAST</stp>
         <tr r="B5" s="2"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>Last Price</v>
         <stp/>
         <stp>##V3_BFIELDINFOV12</stp>
         <stp>[Gas storages.xlsx]Prices!R5C3</stp>
         <stp>PX_LAST</stp>
         <tr r="C5" s="2"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>Last Price</v>
         <stp/>
         <stp>##V3_BFIELDINFOV12</stp>
         <stp>[Gas storages.xlsx]Stocks!R5C4</stp>
         <stp>PX_LAST</stp>
         <tr r="D5" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>Last Price</v>
         <stp/>
         <stp>##V3_BFIELDINFOV12</stp>
         <stp>[Gas storages.xlsx]Stocks!R5C5</stp>
         <stp>PX_LAST</stp>
         <tr r="E5" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>Last Price</v>
         <stp/>
         <stp>##V3_BFIELDINFOV12</stp>
         <stp>[Gas storages.xlsx]Stocks!R5C6</stp>
         <stp>PX_LAST</stp>
         <tr r="F5" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>Last Price</v>
         <stp/>
         <stp>##V3_BFIELDINFOV12</stp>
         <stp>[Gas storages.xlsx]Stocks!R5C2</stp>
         <stp>PX_LAST</stp>
         <tr r="B5" s="1"/>
       </tp>
-      <tp t="e">
-        <v>#N/A</v>
+      <tp t="s">
+        <v>Last Price</v>
         <stp/>
         <stp>##V3_BFIELDINFOV12</stp>
         <stp>[Gas storages.xlsx]Stocks!R5C3</stp>
@@ -254,8 +254,8 @@
         <v>#N/A</v>
         <stp/>
         <stp>BDH|5828156284080324637</stp>
+        <tr r="A7" s="2"/>
         <tr r="A7" s="3"/>
-        <tr r="A7" s="2"/>
       </tp>
       <tp t="e">
         <v>#N/A</v>
@@ -263,6 +263,8 @@
         <stp>BDH|1378406766753827437</stp>
         <tr r="C7" s="3"/>
       </tp>
+    </main>
+    <main first="bofaddin.rtdserver">
       <tp t="e">
         <v>#N/A</v>
         <stp/>
@@ -623,7 +625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3900AD71-E3B4-44B6-951D-A8605D5D6C7F}">
-  <dimension ref="A1:F1459"/>
+  <dimension ref="A1:F1475"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
@@ -725,26 +727,26 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
-        <f>_xll.BDH(B$4,B$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S","cols=2;rows=1453")</f>
+        <f>_xll.BDH(B$4,B$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S","cols=2;rows=1469")</f>
         <v>43831</v>
       </c>
       <c r="B7">
         <v>990.32669999999996</v>
       </c>
       <c r="C7">
-        <f>_xll.BDH(C$4,C$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1453")</f>
+        <f>_xll.BDH(C$4,C$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1469")</f>
         <v>3192</v>
       </c>
       <c r="D7">
-        <f>_xll.BDH(D$4,D$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1453")</f>
+        <f>_xll.BDH(D$4,D$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1469")</f>
         <v>11.5663</v>
       </c>
       <c r="E7">
-        <f>_xll.BDH(E$4,E$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1453")</f>
+        <f>_xll.BDH(E$4,E$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1469")</f>
         <v>233.00030000000001</v>
       </c>
       <c r="F7">
-        <f>_xll.BDH(F$4,F$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1453")</f>
+        <f>_xll.BDH(F$4,F$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1469")</f>
         <v>107.5916</v>
       </c>
     </row>
@@ -28493,7 +28495,7 @@
         <v>45775</v>
       </c>
       <c r="B1395">
-        <v>440.1164</v>
+        <v>440.11750000000001</v>
       </c>
       <c r="C1395">
         <v>2041</v>
@@ -28513,7 +28515,7 @@
         <v>45776</v>
       </c>
       <c r="B1396">
-        <v>443.06229999999999</v>
+        <v>443.06630000000001</v>
       </c>
       <c r="C1396">
         <v>2041</v>
@@ -28533,7 +28535,7 @@
         <v>45777</v>
       </c>
       <c r="B1397">
-        <v>446.488</v>
+        <v>446.49369999999999</v>
       </c>
       <c r="C1397">
         <v>2041</v>
@@ -28553,7 +28555,7 @@
         <v>45778</v>
       </c>
       <c r="B1398">
-        <v>451.06909999999999</v>
+        <v>451.07470000000001</v>
       </c>
       <c r="C1398">
         <v>2041</v>
@@ -28573,7 +28575,7 @@
         <v>45779</v>
       </c>
       <c r="B1399">
-        <v>455.56639999999999</v>
+        <v>455.57459999999998</v>
       </c>
       <c r="C1399">
         <v>2145</v>
@@ -28593,7 +28595,7 @@
         <v>45782</v>
       </c>
       <c r="B1400">
-        <v>468.04610000000002</v>
+        <v>468.05799999999999</v>
       </c>
       <c r="C1400">
         <v>2145</v>
@@ -28613,7 +28615,7 @@
         <v>45783</v>
       </c>
       <c r="B1401">
-        <v>470.5521</v>
+        <v>470.56549999999999</v>
       </c>
       <c r="C1401">
         <v>2145</v>
@@ -28633,7 +28635,7 @@
         <v>45784</v>
       </c>
       <c r="B1402">
-        <v>472.851</v>
+        <v>472.86439999999999</v>
       </c>
       <c r="C1402">
         <v>2145</v>
@@ -28973,7 +28975,7 @@
         <v>45807</v>
       </c>
       <c r="B1419">
-        <v>542.30190000000005</v>
+        <v>542.30200000000002</v>
       </c>
       <c r="C1419">
         <v>2598</v>
@@ -28993,7 +28995,7 @@
         <v>45810</v>
       </c>
       <c r="B1420">
-        <v>558.1413</v>
+        <v>558.14120000000003</v>
       </c>
       <c r="C1420">
         <v>2598</v>
@@ -29005,7 +29007,7 @@
         <v>102.35120000000001</v>
       </c>
       <c r="F1420">
-        <v>53.1571</v>
+        <v>53.156999999999996</v>
       </c>
     </row>
     <row r="1421" spans="1:6" x14ac:dyDescent="0.25">
@@ -29053,7 +29055,7 @@
         <v>45813</v>
       </c>
       <c r="B1423">
-        <v>568.90740000000005</v>
+        <v>568.90689999999995</v>
       </c>
       <c r="C1423">
         <v>2598</v>
@@ -29065,7 +29067,7 @@
         <v>104.0763</v>
       </c>
       <c r="F1423">
-        <v>54.804499999999997</v>
+        <v>54.804099999999998</v>
       </c>
     </row>
     <row r="1424" spans="1:6" x14ac:dyDescent="0.25">
@@ -29073,7 +29075,7 @@
         <v>45814</v>
       </c>
       <c r="B1424">
-        <v>573.02679999999998</v>
+        <v>573.02480000000003</v>
       </c>
       <c r="C1424">
         <v>2707</v>
@@ -29085,7 +29087,7 @@
         <v>104.97580000000001</v>
       </c>
       <c r="F1424">
-        <v>55.370800000000003</v>
+        <v>55.3688</v>
       </c>
     </row>
     <row r="1425" spans="1:6" x14ac:dyDescent="0.25">
@@ -29093,7 +29095,7 @@
         <v>45817</v>
       </c>
       <c r="B1425">
-        <v>587.34019999999998</v>
+        <v>587.33709999999996</v>
       </c>
       <c r="C1425">
         <v>2707</v>
@@ -29105,7 +29107,7 @@
         <v>108.14190000000001</v>
       </c>
       <c r="F1425">
-        <v>57.259799999999998</v>
+        <v>57.256700000000002</v>
       </c>
     </row>
     <row r="1426" spans="1:6" x14ac:dyDescent="0.25">
@@ -29113,7 +29115,7 @@
         <v>45818</v>
       </c>
       <c r="B1426">
-        <v>591.0675</v>
+        <v>591.06859999999995</v>
       </c>
       <c r="C1426">
         <v>2707</v>
@@ -29125,7 +29127,7 @@
         <v>108.9713</v>
       </c>
       <c r="F1426">
-        <v>57.725099999999998</v>
+        <v>57.726199999999999</v>
       </c>
     </row>
     <row r="1427" spans="1:6" x14ac:dyDescent="0.25">
@@ -29133,7 +29135,7 @@
         <v>45819</v>
       </c>
       <c r="B1427">
-        <v>594.70830000000001</v>
+        <v>594.70979999999997</v>
       </c>
       <c r="C1427">
         <v>2707</v>
@@ -29145,7 +29147,7 @@
         <v>109.6807</v>
       </c>
       <c r="F1427">
-        <v>58.259700000000002</v>
+        <v>58.261299999999999</v>
       </c>
     </row>
     <row r="1428" spans="1:6" x14ac:dyDescent="0.25">
@@ -29153,7 +29155,7 @@
         <v>45820</v>
       </c>
       <c r="B1428">
-        <v>598.19539999999995</v>
+        <v>598.197</v>
       </c>
       <c r="C1428">
         <v>2707</v>
@@ -29165,7 +29167,7 @@
         <v>110.3668</v>
       </c>
       <c r="F1428">
-        <v>58.807499999999997</v>
+        <v>58.809100000000001</v>
       </c>
     </row>
     <row r="1429" spans="1:6" x14ac:dyDescent="0.25">
@@ -29173,7 +29175,7 @@
         <v>45821</v>
       </c>
       <c r="B1429">
-        <v>601.23199999999997</v>
+        <v>601.23360000000002</v>
       </c>
       <c r="C1429">
         <v>2802</v>
@@ -29185,7 +29187,7 @@
         <v>111.04900000000001</v>
       </c>
       <c r="F1429">
-        <v>59.381500000000003</v>
+        <v>59.383099999999999</v>
       </c>
     </row>
     <row r="1430" spans="1:6" x14ac:dyDescent="0.25">
@@ -29193,7 +29195,7 @@
         <v>45824</v>
       </c>
       <c r="B1430">
-        <v>613.17269999999996</v>
+        <v>613.17420000000004</v>
       </c>
       <c r="C1430">
         <v>2802</v>
@@ -29205,7 +29207,7 @@
         <v>113.9349</v>
       </c>
       <c r="F1430">
-        <v>61.184899999999999</v>
+        <v>61.186500000000002</v>
       </c>
     </row>
     <row r="1431" spans="1:6" x14ac:dyDescent="0.25">
@@ -29213,7 +29215,7 @@
         <v>45825</v>
       </c>
       <c r="B1431">
-        <v>616.73009999999999</v>
+        <v>616.73159999999996</v>
       </c>
       <c r="C1431">
         <v>2802</v>
@@ -29225,7 +29227,7 @@
         <v>114.5381</v>
       </c>
       <c r="F1431">
-        <v>61.7376</v>
+        <v>61.739199999999997</v>
       </c>
     </row>
     <row r="1432" spans="1:6" x14ac:dyDescent="0.25">
@@ -29233,7 +29235,7 @@
         <v>45826</v>
       </c>
       <c r="B1432">
-        <v>620.50660000000005</v>
+        <v>620.50819999999999</v>
       </c>
       <c r="C1432">
         <v>2802</v>
@@ -29245,7 +29247,7 @@
         <v>115.23560000000001</v>
       </c>
       <c r="F1432">
-        <v>62.357100000000003</v>
+        <v>62.358699999999999</v>
       </c>
     </row>
     <row r="1433" spans="1:6" x14ac:dyDescent="0.25">
@@ -29253,7 +29255,7 @@
         <v>45827</v>
       </c>
       <c r="B1433">
-        <v>624.35450000000003</v>
+        <v>624.35599999999999</v>
       </c>
       <c r="C1433">
         <v>2802</v>
@@ -29265,7 +29267,7 @@
         <v>116.04640000000001</v>
       </c>
       <c r="F1433">
-        <v>62.974699999999999</v>
+        <v>62.976199999999999</v>
       </c>
     </row>
     <row r="1434" spans="1:6" x14ac:dyDescent="0.25">
@@ -29273,7 +29275,7 @@
         <v>45828</v>
       </c>
       <c r="B1434">
-        <v>628.22239999999999</v>
+        <v>628.22400000000005</v>
       </c>
       <c r="C1434">
         <v>2898</v>
@@ -29285,7 +29287,7 @@
         <v>116.8073</v>
       </c>
       <c r="F1434">
-        <v>63.595199999999998</v>
+        <v>63.596699999999998</v>
       </c>
     </row>
     <row r="1435" spans="1:6" x14ac:dyDescent="0.25">
@@ -29293,7 +29295,7 @@
         <v>45831</v>
       </c>
       <c r="B1435">
-        <v>641.81209999999999</v>
+        <v>641.75149999999996</v>
       </c>
       <c r="C1435">
         <v>2898</v>
@@ -29305,7 +29307,7 @@
         <v>119.9722</v>
       </c>
       <c r="F1435">
-        <v>65.188299999999998</v>
+        <v>65.189800000000005</v>
       </c>
     </row>
     <row r="1436" spans="1:6" x14ac:dyDescent="0.25">
@@ -29313,7 +29315,7 @@
         <v>45832</v>
       </c>
       <c r="B1436">
-        <v>645.34460000000001</v>
+        <v>645.34619999999995</v>
       </c>
       <c r="C1436">
         <v>2898</v>
@@ -29325,7 +29327,7 @@
         <v>120.7569</v>
       </c>
       <c r="F1436">
-        <v>65.6965</v>
+        <v>65.698099999999997</v>
       </c>
     </row>
     <row r="1437" spans="1:6" x14ac:dyDescent="0.25">
@@ -29333,7 +29335,7 @@
         <v>45833</v>
       </c>
       <c r="B1437">
-        <v>648.32280000000003</v>
+        <v>648.32439999999997</v>
       </c>
       <c r="C1437">
         <v>2898</v>
@@ -29345,7 +29347,7 @@
         <v>121.1504</v>
       </c>
       <c r="F1437">
-        <v>66.267899999999997</v>
+        <v>66.269400000000005</v>
       </c>
     </row>
     <row r="1438" spans="1:6" x14ac:dyDescent="0.25">
@@ -29353,7 +29355,7 @@
         <v>45834</v>
       </c>
       <c r="B1438">
-        <v>651.19230000000005</v>
+        <v>651.19389999999999</v>
       </c>
       <c r="C1438">
         <v>2898</v>
@@ -29365,7 +29367,7 @@
         <v>121.288</v>
       </c>
       <c r="F1438">
-        <v>66.8797</v>
+        <v>66.881200000000007</v>
       </c>
     </row>
     <row r="1439" spans="1:6" x14ac:dyDescent="0.25">
@@ -29373,7 +29375,7 @@
         <v>45835</v>
       </c>
       <c r="B1439">
-        <v>655.18119999999999</v>
+        <v>655.18280000000004</v>
       </c>
       <c r="C1439">
         <v>2953</v>
@@ -29385,7 +29387,7 @@
         <v>122.3229</v>
       </c>
       <c r="F1439">
-        <v>67.494600000000005</v>
+        <v>67.496200000000002</v>
       </c>
     </row>
     <row r="1440" spans="1:6" x14ac:dyDescent="0.25">
@@ -29393,7 +29395,7 @@
         <v>45838</v>
       </c>
       <c r="B1440">
-        <v>667.93299999999999</v>
+        <v>667.93449999999996</v>
       </c>
       <c r="C1440">
         <v>2953</v>
@@ -29405,7 +29407,7 @@
         <v>125.3109</v>
       </c>
       <c r="F1440">
-        <v>69.207899999999995</v>
+        <v>69.209400000000002</v>
       </c>
     </row>
     <row r="1441" spans="1:6" x14ac:dyDescent="0.25">
@@ -29413,7 +29415,7 @@
         <v>45839</v>
       </c>
       <c r="B1441">
-        <v>670.72990000000004</v>
+        <v>670.73140000000001</v>
       </c>
       <c r="C1441">
         <v>2953</v>
@@ -29425,7 +29427,7 @@
         <v>125.98990000000001</v>
       </c>
       <c r="F1441">
-        <v>69.485399999999998</v>
+        <v>69.486999999999995</v>
       </c>
     </row>
     <row r="1442" spans="1:6" x14ac:dyDescent="0.25">
@@ -29493,7 +29495,7 @@
         <v>45845</v>
       </c>
       <c r="B1445">
-        <v>694.87829999999997</v>
+        <v>691.0444</v>
       </c>
       <c r="C1445">
         <v>3006</v>
@@ -29502,7 +29504,7 @@
         <v>2.6970000000000001</v>
       </c>
       <c r="E1445">
-        <v>134.70599999999999</v>
+        <v>130.87200000000001</v>
       </c>
       <c r="F1445">
         <v>71.979699999999994</v>
@@ -29513,7 +29515,7 @@
         <v>45846</v>
       </c>
       <c r="B1446">
-        <v>698.37159999999994</v>
+        <v>698.37090000000001</v>
       </c>
       <c r="C1446">
         <v>3006</v>
@@ -29533,7 +29535,7 @@
         <v>45847</v>
       </c>
       <c r="B1447">
-        <v>698.08040000000005</v>
+        <v>698.08</v>
       </c>
       <c r="C1447">
         <v>3006</v>
@@ -29553,7 +29555,7 @@
         <v>45848</v>
       </c>
       <c r="B1448">
-        <v>701.96960000000001</v>
+        <v>702.0018</v>
       </c>
       <c r="C1448">
         <v>3006</v>
@@ -29573,7 +29575,7 @@
         <v>45849</v>
       </c>
       <c r="B1449">
-        <v>705.5598</v>
+        <v>705.6327</v>
       </c>
       <c r="C1449">
         <v>3052</v>
@@ -29713,7 +29715,7 @@
         <v>45860</v>
       </c>
       <c r="B1456">
-        <v>745.10479999999995</v>
+        <v>745.11170000000004</v>
       </c>
       <c r="C1456">
         <v>3075</v>
@@ -29733,7 +29735,7 @@
         <v>45861</v>
       </c>
       <c r="B1457">
-        <v>748.33460000000002</v>
+        <v>748.35050000000001</v>
       </c>
       <c r="C1457">
         <v>3075</v>
@@ -29753,7 +29755,7 @@
         <v>45862</v>
       </c>
       <c r="B1458">
-        <v>748.33460000000002</v>
+        <v>751.14070000000004</v>
       </c>
       <c r="C1458">
         <v>3075</v>
@@ -29762,10 +29764,10 @@
         <v>3.0579999999999998</v>
       </c>
       <c r="E1458">
-        <v>143.8321</v>
+        <v>144.21610000000001</v>
       </c>
       <c r="F1458">
-        <v>79.651799999999994</v>
+        <v>80.119900000000001</v>
       </c>
     </row>
     <row r="1459" spans="1:6" x14ac:dyDescent="0.25">
@@ -29773,19 +29775,339 @@
         <v>45863</v>
       </c>
       <c r="B1459">
-        <v>748.33460000000002</v>
+        <v>754.31640000000004</v>
       </c>
       <c r="C1459">
-        <v>3075</v>
+        <v>3123</v>
       </c>
       <c r="D1459">
-        <v>3.0579999999999998</v>
+        <v>3.1030000000000002</v>
       </c>
       <c r="E1459">
-        <v>143.8321</v>
+        <v>144.81639999999999</v>
       </c>
       <c r="F1459">
-        <v>79.651799999999994</v>
+        <v>80.617999999999995</v>
+      </c>
+    </row>
+    <row r="1460" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1460" s="2">
+        <v>45866</v>
+      </c>
+      <c r="B1460">
+        <v>766.94910000000004</v>
+      </c>
+      <c r="C1460">
+        <v>3123</v>
+      </c>
+      <c r="D1460">
+        <v>3.2551999999999999</v>
+      </c>
+      <c r="E1460">
+        <v>147.88030000000001</v>
+      </c>
+      <c r="F1460">
+        <v>82.192300000000003</v>
+      </c>
+    </row>
+    <row r="1461" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1461" s="2">
+        <v>45867</v>
+      </c>
+      <c r="B1461">
+        <v>771.0367</v>
+      </c>
+      <c r="C1461">
+        <v>3123</v>
+      </c>
+      <c r="D1461">
+        <v>3.3001999999999998</v>
+      </c>
+      <c r="E1461">
+        <v>148.80629999999999</v>
+      </c>
+      <c r="F1461">
+        <v>82.695300000000003</v>
+      </c>
+    </row>
+    <row r="1462" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1462" s="2">
+        <v>45868</v>
+      </c>
+      <c r="B1462">
+        <v>774.92340000000002</v>
+      </c>
+      <c r="C1462">
+        <v>3123</v>
+      </c>
+      <c r="D1462">
+        <v>3.3599000000000001</v>
+      </c>
+      <c r="E1462">
+        <v>149.7362</v>
+      </c>
+      <c r="F1462">
+        <v>83.131500000000003</v>
+      </c>
+    </row>
+    <row r="1463" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1463" s="2">
+        <v>45869</v>
+      </c>
+      <c r="B1463">
+        <v>778.27629999999999</v>
+      </c>
+      <c r="C1463">
+        <v>3123</v>
+      </c>
+      <c r="D1463">
+        <v>3.4049</v>
+      </c>
+      <c r="E1463">
+        <v>150.3691</v>
+      </c>
+      <c r="F1463">
+        <v>83.5411</v>
+      </c>
+    </row>
+    <row r="1464" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1464" s="2">
+        <v>45870</v>
+      </c>
+      <c r="B1464">
+        <v>781.83960000000002</v>
+      </c>
+      <c r="C1464">
+        <v>3130</v>
+      </c>
+      <c r="D1464">
+        <v>3.4657</v>
+      </c>
+      <c r="E1464">
+        <v>151.13319999999999</v>
+      </c>
+      <c r="F1464">
+        <v>83.945300000000003</v>
+      </c>
+    </row>
+    <row r="1465" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1465" s="2">
+        <v>45873</v>
+      </c>
+      <c r="B1465">
+        <v>794.49419999999998</v>
+      </c>
+      <c r="C1465">
+        <v>3130</v>
+      </c>
+      <c r="D1465">
+        <v>3.6278000000000001</v>
+      </c>
+      <c r="E1465">
+        <v>154.71690000000001</v>
+      </c>
+      <c r="F1465">
+        <v>85.112499999999997</v>
+      </c>
+    </row>
+    <row r="1466" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1466" s="2">
+        <v>45874</v>
+      </c>
+      <c r="B1466">
+        <v>798.28729999999996</v>
+      </c>
+      <c r="C1466">
+        <v>3130</v>
+      </c>
+      <c r="D1466">
+        <v>3.8363</v>
+      </c>
+      <c r="E1466">
+        <v>155.80699999999999</v>
+      </c>
+      <c r="F1466">
+        <v>85.433899999999994</v>
+      </c>
+    </row>
+    <row r="1467" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1467" s="2">
+        <v>45875</v>
+      </c>
+      <c r="B1467">
+        <v>801.97329999999999</v>
+      </c>
+      <c r="C1467">
+        <v>3130</v>
+      </c>
+      <c r="D1467">
+        <v>3.944</v>
+      </c>
+      <c r="E1467">
+        <v>156.71440000000001</v>
+      </c>
+      <c r="F1467">
+        <v>85.705600000000004</v>
+      </c>
+    </row>
+    <row r="1468" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1468" s="2">
+        <v>45876</v>
+      </c>
+      <c r="B1468">
+        <v>805.52599999999995</v>
+      </c>
+      <c r="C1468">
+        <v>3130</v>
+      </c>
+      <c r="D1468">
+        <v>4.0647000000000002</v>
+      </c>
+      <c r="E1468">
+        <v>157.53829999999999</v>
+      </c>
+      <c r="F1468">
+        <v>86.035200000000003</v>
+      </c>
+    </row>
+    <row r="1469" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1469" s="2">
+        <v>45877</v>
+      </c>
+      <c r="B1469">
+        <v>809.06349999999998</v>
+      </c>
+      <c r="C1469">
+        <v>3186</v>
+      </c>
+      <c r="D1469">
+        <v>4.1501999999999999</v>
+      </c>
+      <c r="E1469">
+        <v>158.38079999999999</v>
+      </c>
+      <c r="F1469">
+        <v>86.459299999999999</v>
+      </c>
+    </row>
+    <row r="1470" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1470" s="2">
+        <v>45880</v>
+      </c>
+      <c r="B1470">
+        <v>820.99189999999999</v>
+      </c>
+      <c r="C1470">
+        <v>3186</v>
+      </c>
+      <c r="D1470">
+        <v>4.4446000000000003</v>
+      </c>
+      <c r="E1470">
+        <v>161.44370000000001</v>
+      </c>
+      <c r="F1470">
+        <v>87.696299999999994</v>
+      </c>
+    </row>
+    <row r="1471" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1471" s="2">
+        <v>45881</v>
+      </c>
+      <c r="B1471">
+        <v>823.96029999999996</v>
+      </c>
+      <c r="C1471">
+        <v>3186</v>
+      </c>
+      <c r="D1471">
+        <v>4.4355000000000002</v>
+      </c>
+      <c r="E1471">
+        <v>162.1422</v>
+      </c>
+      <c r="F1471">
+        <v>87.944100000000006</v>
+      </c>
+    </row>
+    <row r="1472" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1472" s="2">
+        <v>45882</v>
+      </c>
+      <c r="B1472">
+        <v>826.71749999999997</v>
+      </c>
+      <c r="C1472">
+        <v>3186</v>
+      </c>
+      <c r="D1472">
+        <v>4.4782999999999999</v>
+      </c>
+      <c r="E1472">
+        <v>162.76599999999999</v>
+      </c>
+      <c r="F1472">
+        <v>88.168599999999998</v>
+      </c>
+    </row>
+    <row r="1473" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1473" s="2">
+        <v>45883</v>
+      </c>
+      <c r="B1473">
+        <v>829.09180000000003</v>
+      </c>
+      <c r="C1473">
+        <v>3186</v>
+      </c>
+      <c r="D1473">
+        <v>4.5212000000000003</v>
+      </c>
+      <c r="E1473">
+        <v>163.50049999999999</v>
+      </c>
+      <c r="F1473">
+        <v>88.382400000000004</v>
+      </c>
+    </row>
+    <row r="1474" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1474" s="2">
+        <v>45884</v>
+      </c>
+      <c r="B1474">
+        <v>832.59289999999999</v>
+      </c>
+      <c r="C1474">
+        <v>3186</v>
+      </c>
+      <c r="D1474">
+        <v>4.5640000000000001</v>
+      </c>
+      <c r="E1474">
+        <v>164.47280000000001</v>
+      </c>
+      <c r="F1474">
+        <v>88.7393</v>
+      </c>
+    </row>
+    <row r="1475" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1475" s="2">
+        <v>45887</v>
+      </c>
+      <c r="B1475">
+        <v>836.16790000000003</v>
+      </c>
+      <c r="C1475">
+        <v>3186</v>
+      </c>
+      <c r="D1475">
+        <v>4.5944000000000003</v>
+      </c>
+      <c r="E1475">
+        <v>165.3801</v>
+      </c>
+      <c r="F1475">
+        <v>89.182400000000001</v>
       </c>
     </row>
   </sheetData>
@@ -29795,7 +30117,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9CC2F69-7C8C-4154-8046-9289F76718B0}">
-  <dimension ref="A1:C1197"/>
+  <dimension ref="A1:C1213"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -29847,14 +30169,14 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
-        <f>_xll.BDH(B$4,B$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S","cols=2;rows=1191")</f>
+        <f>_xll.BDH(B$4,B$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=S","cols=2;rows=1207")</f>
         <v>44197</v>
       </c>
       <c r="B7">
         <v>32.590000000000003</v>
       </c>
       <c r="C7">
-        <f>_xll.BDH(C$4,C$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1191")</f>
+        <f>_xll.BDH(C$4,C$6,$B1,$B2,"Dir=V","CDR=5D","Days=A","Dts=H","cols=1;rows=1207")</f>
         <v>19.074999999999999</v>
       </c>
     </row>
@@ -42942,10 +43264,186 @@
         <v>45863</v>
       </c>
       <c r="B1197">
-        <v>70.63</v>
+        <v>70.959999999999994</v>
       </c>
       <c r="C1197">
-        <v>32.549999999999997</v>
+        <v>32.43</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1198" s="2">
+        <v>45866</v>
+      </c>
+      <c r="B1198">
+        <v>70.27</v>
+      </c>
+      <c r="C1198">
+        <v>33.049999999999997</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1199" s="2">
+        <v>45867</v>
+      </c>
+      <c r="B1199">
+        <v>72.680000000000007</v>
+      </c>
+      <c r="C1199">
+        <v>34.18</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1200" s="2">
+        <v>45868</v>
+      </c>
+      <c r="B1200">
+        <v>72.459999999999994</v>
+      </c>
+      <c r="C1200">
+        <v>34.4</v>
+      </c>
+    </row>
+    <row r="1201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1201" s="2">
+        <v>45869</v>
+      </c>
+      <c r="B1201">
+        <v>72.25</v>
+      </c>
+      <c r="C1201">
+        <v>34.549999999999997</v>
+      </c>
+    </row>
+    <row r="1202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1202" s="2">
+        <v>45870</v>
+      </c>
+      <c r="B1202">
+        <v>70.66</v>
+      </c>
+      <c r="C1202">
+        <v>33.774999999999999</v>
+      </c>
+    </row>
+    <row r="1203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1203" s="2">
+        <v>45873</v>
+      </c>
+      <c r="B1203">
+        <v>70.459999999999994</v>
+      </c>
+      <c r="C1203">
+        <v>34.15</v>
+      </c>
+    </row>
+    <row r="1204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1204" s="2">
+        <v>45874</v>
+      </c>
+      <c r="B1204">
+        <v>71.2</v>
+      </c>
+      <c r="C1204">
+        <v>34.35</v>
+      </c>
+    </row>
+    <row r="1205" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1205" s="2">
+        <v>45875</v>
+      </c>
+      <c r="B1205">
+        <v>70.599999999999994</v>
+      </c>
+      <c r="C1205">
+        <v>33.25</v>
+      </c>
+    </row>
+    <row r="1206" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1206" s="2">
+        <v>45876</v>
+      </c>
+      <c r="B1206">
+        <v>71.38</v>
+      </c>
+      <c r="C1206">
+        <v>33.024999999999999</v>
+      </c>
+    </row>
+    <row r="1207" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1207" s="2">
+        <v>45877</v>
+      </c>
+      <c r="B1207">
+        <v>72.81</v>
+      </c>
+      <c r="C1207">
+        <v>32.174999999999997</v>
+      </c>
+    </row>
+    <row r="1208" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1208" s="2">
+        <v>45880</v>
+      </c>
+      <c r="B1208">
+        <v>71.98</v>
+      </c>
+      <c r="C1208">
+        <v>33.125</v>
+      </c>
+    </row>
+    <row r="1209" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1209" s="2">
+        <v>45881</v>
+      </c>
+      <c r="B1209">
+        <v>71.12</v>
+      </c>
+      <c r="C1209">
+        <v>32.450000000000003</v>
+      </c>
+    </row>
+    <row r="1210" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1210" s="2">
+        <v>45882</v>
+      </c>
+      <c r="B1210">
+        <v>71.349999999999994</v>
+      </c>
+      <c r="C1210">
+        <v>32.68</v>
+      </c>
+    </row>
+    <row r="1211" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1211" s="2">
+        <v>45883</v>
+      </c>
+      <c r="B1211">
+        <v>70.569999999999993</v>
+      </c>
+      <c r="C1211">
+        <v>32.229999999999997</v>
+      </c>
+    </row>
+    <row r="1212" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1212" s="2">
+        <v>45884</v>
+      </c>
+      <c r="B1212">
+        <v>70.3</v>
+      </c>
+      <c r="C1212">
+        <v>30.88</v>
+      </c>
+    </row>
+    <row r="1213" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1213" s="2">
+        <v>45887</v>
+      </c>
+      <c r="B1213">
+        <v>70.5</v>
+      </c>
+      <c r="C1213">
+        <v>30.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>